<commit_message>
Mark Acid Wash medium out of stock
</commit_message>
<xml_diff>
--- a/Business/out-of-stock.xlsx
+++ b/Business/out-of-stock.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\Denied\Business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C45501-97B7-4911-B94B-5324A33E6F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F4F408D-4571-40A6-ACB6-8E49BA4191B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="21">
   <si>
     <t>S.No.</t>
   </si>
@@ -93,6 +93,12 @@
   </si>
   <si>
     <t>XS</t>
+  </si>
+  <si>
+    <t>Acid Washed</t>
+  </si>
+  <si>
+    <t>Black</t>
   </si>
 </sst>
 </file>
@@ -430,12 +436,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
     <col min="2" max="2" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="8.88671875" style="1"/>
   </cols>
@@ -530,7 +536,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <f t="shared" ref="A6:A10" si="0">A5+1</f>
+        <f t="shared" ref="A6:A11" si="0">A5+1</f>
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -618,6 +624,24 @@
         <v>18</v>
       </c>
     </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh out-of-stock variants from supplier sheet
</commit_message>
<xml_diff>
--- a/Business/out-of-stock.xlsx
+++ b/Business/out-of-stock.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\Denied\Business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F4F408D-4571-40A6-ACB6-8E49BA4191B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8755524-5515-434E-A2D5-03ED0AD2D567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="23">
   <si>
     <t>S.No.</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Coffee Brown</t>
   </si>
   <si>
-    <t>Brick Red</t>
-  </si>
-  <si>
     <t>L</t>
   </si>
   <si>
@@ -80,15 +77,9 @@
     <t>Oversized</t>
   </si>
   <si>
-    <t>Royal Blue</t>
-  </si>
-  <si>
     <t>Olive Green</t>
   </si>
   <si>
-    <t>XXL</t>
-  </si>
-  <si>
     <t>S</t>
   </si>
   <si>
@@ -99,6 +90,21 @@
   </si>
   <si>
     <t>Black</t>
+  </si>
+  <si>
+    <t>XXXL</t>
+  </si>
+  <si>
+    <t>Maroon</t>
+  </si>
+  <si>
+    <t>Light Baby Pink</t>
+  </si>
+  <si>
+    <t>Lavender</t>
+  </si>
+  <si>
+    <t>White</t>
   </si>
 </sst>
 </file>
@@ -436,7 +442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -474,10 +480,10 @@
         <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -492,10 +498,10 @@
         <v>6</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -504,16 +510,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -522,31 +528,31 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <f t="shared" ref="A6:A11" si="0">A5+1</f>
+        <f t="shared" ref="A6:A13" si="0">A5+1</f>
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>9</v>
@@ -558,16 +564,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -576,16 +582,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -594,16 +600,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -612,16 +618,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -630,15 +636,51 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct stock mapping for Moody Floaty variants
</commit_message>
<xml_diff>
--- a/Business/out-of-stock.xlsx
+++ b/Business/out-of-stock.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\Denied\Business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8755524-5515-434E-A2D5-03ED0AD2D567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C702A0-8B95-4E4A-9DE7-D5A0A505FD38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -92,9 +92,6 @@
     <t>Black</t>
   </si>
   <si>
-    <t>XXXL</t>
-  </si>
-  <si>
     <t>Maroon</t>
   </si>
   <si>
@@ -105,6 +102,9 @@
   </si>
   <si>
     <t>White</t>
+  </si>
+  <si>
+    <t>3XL</t>
   </si>
 </sst>
 </file>
@@ -483,7 +483,7 @@
         <v>17</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -552,7 +552,7 @@
         <v>12</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>9</v>
@@ -618,13 +618,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>9</v>
@@ -636,13 +636,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>9</v>
@@ -660,7 +660,7 @@
         <v>12</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>9</v>
@@ -678,7 +678,7 @@
         <v>12</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>10</v>

</xml_diff>